<commit_message>
Added two new modules, bumped spotbugs and synched from internal repo.
</commit_message>
<xml_diff>
--- a/lib/cumba-oss-cdisc-report-xlsx/src/main/resources/templates/report-template.xlsx
+++ b/lib/cumba-oss-cdisc-report-xlsx/src/main/resources/templates/report-template.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="45">
   <si>
     <t>CORE-ID</t>
   </si>
@@ -156,6 +156,15 @@
   </si>
   <si>
     <t>LOINC Version</t>
+  </si>
+  <si>
+    <t>Dictionary Basis</t>
+  </si>
+  <si>
+    <t>Neoplasm Version</t>
+  </si>
+  <si>
+    <t>Library Metadata Basis</t>
   </si>
 </sst>
 </file>
@@ -641,7 +650,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.109375" bestFit="1" customWidth="1"/>
@@ -781,6 +790,26 @@
       <c r="B20" s="9" t="s">
         <v>35</v>
       </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" s="9"/>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B23" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>